<commit_message>
Add J6 assembly part code
</commit_message>
<xml_diff>
--- a/PCB/Revision 6/PCB Production Files/BOM.xlsx
+++ b/PCB/Revision 6/PCB Production Files/BOM.xlsx
@@ -25,9 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="143">
-  <si>
-    <t xml:space="preserve">Designator</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="144">
+  <si>
+    <t xml:space="preserve">﻿Designator</t>
   </si>
   <si>
     <t xml:space="preserve">Value</t>
@@ -183,16 +183,19 @@
     <t xml:space="preserve">ER-CON06HB-1_Compatible_1x06_P0.50mm_BottomContact</t>
   </si>
   <si>
+    <t xml:space="preserve">C202118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS3625 Module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS3625_Module_Back_Mount_SMD</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">MIC1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS3625 Module</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS3625_Module_Back_Mount_SMD</t>
   </si>
   <si>
     <t xml:space="preserve">Q1,Q3,Q4,Q5,Q7</t>
@@ -462,7 +465,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -498,7 +501,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -817,10 +822,10 @@
   <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="58" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1030,357 +1035,357 @@
         <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D23" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" t="s">
+        <v>89</v>
+      </c>
+      <c r="C25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" t="s">
         <v>87</v>
-      </c>
-      <c r="B25" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D28" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D32" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D34" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B35" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D36" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C37" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B40" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Rev6 JLCPCB assembly files
</commit_message>
<xml_diff>
--- a/PCB/Revision 6/PCB Production Files/BOM.xlsx
+++ b/PCB/Revision 6/PCB Production Files/BOM.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="147">
   <si>
     <t xml:space="preserve">﻿Designator</t>
   </si>
@@ -81,7 +81,7 @@
     <t xml:space="preserve">D_SOD-323</t>
   </si>
   <si>
-    <t xml:space="preserve">C155590</t>
+    <t xml:space="preserve">C49238173</t>
   </si>
   <si>
     <t xml:space="preserve">D2</t>
@@ -457,6 +457,15 @@
   </si>
   <si>
     <t xml:space="preserve">C138713</t>
+  </si>
+  <si>
+    <t>C22765</t>
+  </si>
+  <si>
+    <t>C23162</t>
+  </si>
+  <si>
+    <t>C313912</t>
   </si>
 </sst>
 </file>
@@ -818,8 +827,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -1026,136 +1035,136 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C19" t="s">
         <v>71</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
         <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
         <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B22" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C22" t="s">
         <v>71</v>
       </c>
       <c r="D22" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
       </c>
       <c r="D23" t="s">
-        <v>84</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
         <v>71</v>
@@ -1166,225 +1175,211 @@
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B25" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
         <v>71</v>
       </c>
       <c r="D25" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="D26" t="s">
-        <v>92</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="D27" t="s">
-        <v>96</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="C28" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="D28" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>107</v>
       </c>
       <c r="D30" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D32" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C33" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D33" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B34" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C34" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D34" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C35" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D35" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="D36" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C37" t="s">
-        <v>107</v>
+        <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B38" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D38" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>140</v>
-      </c>
-      <c r="B40" t="s">
-        <v>141</v>
-      </c>
-      <c r="C40" t="s">
-        <v>142</v>
-      </c>
-      <c r="D40" t="s">
         <v>143</v>
       </c>
     </row>

</xml_diff>